<commit_message>
Push outputs from CI/CD (2026-09-04 19:30:31)
</commit_message>
<xml_diff>
--- a/production/watch-PRELIMINARY/Manufacturing/Assembly/ZSWatch-Watch-bom.xlsx
+++ b/production/watch-PRELIMINARY/Manufacturing/Assembly/ZSWatch-Watch-bom.xlsx
@@ -291,7 +291,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="272">
   <si>
     <t>Row</t>
   </si>
@@ -647,6 +647,24 @@
     <t>19</t>
   </si>
   <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>53261-0271</t>
+  </si>
+  <si>
+    <t>https://www.molex.com/pdm_docs/sd/532610271_sd.pdf</t>
+  </si>
+  <si>
+    <t>molex_pico</t>
+  </si>
+  <si>
+    <t>1.25mm Pitch, PicoBlade PCB Header, Single Row, Right-Angle, Surface Mount, Tin (Sn) Plating, Friction Lock,  Circuits, Tape and Reel</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
     <t>L401 L402</t>
   </si>
   <si>
@@ -662,7 +680,7 @@
     <t>LQM18PZ2R2MDHD</t>
   </si>
   <si>
-    <t>20</t>
+    <t>21</t>
   </si>
   <si>
     <t>LS801</t>
@@ -680,7 +698,7 @@
     <t>Same Sky</t>
   </si>
   <si>
-    <t>21</t>
+    <t>22</t>
   </si>
   <si>
     <t>M601</t>
@@ -698,7 +716,7 @@
     <t>NORA-B106-00B</t>
   </si>
   <si>
-    <t>22</t>
+    <t>23</t>
   </si>
   <si>
     <t>MK501</t>
@@ -716,7 +734,7 @@
     <t>Knowles</t>
   </si>
   <si>
-    <t>23</t>
+    <t>24</t>
   </si>
   <si>
     <t>R501 R502</t>
@@ -740,7 +758,7 @@
     <t>RC0201JR-071K8L</t>
   </si>
   <si>
-    <t>24</t>
+    <t>25</t>
   </si>
   <si>
     <t>R504 R505</t>
@@ -752,7 +770,7 @@
     <t>RC0201JR-073K3L</t>
   </si>
   <si>
-    <t>25</t>
+    <t>26</t>
   </si>
   <si>
     <t>R601</t>
@@ -764,7 +782,7 @@
     <t>RC0201JR-0712KL</t>
   </si>
   <si>
-    <t>26</t>
+    <t>27</t>
   </si>
   <si>
     <t>R407</t>
@@ -776,7 +794,7 @@
     <t>RC0201JR-0747KL</t>
   </si>
   <si>
-    <t>27</t>
+    <t>28</t>
   </si>
   <si>
     <t>R408 R613</t>
@@ -788,7 +806,7 @@
     <t>RC0201JR-07100KL</t>
   </si>
   <si>
-    <t>28</t>
+    <t>29</t>
   </si>
   <si>
     <t>R506</t>
@@ -800,7 +818,7 @@
     <t>RC0201JR-07200KL</t>
   </si>
   <si>
-    <t>29</t>
+    <t>30</t>
   </si>
   <si>
     <t>S501</t>
@@ -824,7 +842,7 @@
     <t>436333033816</t>
   </si>
   <si>
-    <t>30</t>
+    <t>31</t>
   </si>
   <si>
     <t>S502</t>
@@ -833,7 +851,7 @@
     <t>SW2</t>
   </si>
   <si>
-    <t>31</t>
+    <t>32</t>
   </si>
   <si>
     <t>S503</t>
@@ -842,7 +860,7 @@
     <t>SW3</t>
   </si>
   <si>
-    <t>32</t>
+    <t>33</t>
   </si>
   <si>
     <t>S504</t>
@@ -851,111 +869,90 @@
     <t>SW4</t>
   </si>
   <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>X402</t>
-  </si>
-  <si>
-    <t>Battery</t>
-  </si>
-  <si>
-    <t>https://www.mouser.com/catalog/specsheets/JST_SM02B-SRSS-TB_LF_SN_eSR_SZ.pdf</t>
-  </si>
-  <si>
-    <t>JST_SH_SM02B-SRSS-TB_1x02-1MP_P1.00mm_Horizontal</t>
+    <t>34</t>
+  </si>
+  <si>
+    <t>X603</t>
+  </si>
+  <si>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>https://www.usb.org/sites/default/files/documents/usb_type-c.zip</t>
+  </si>
+  <si>
+    <t>USB_C_Receptacle_Amphenol_12401610E4-2A</t>
+  </si>
+  <si>
+    <t>USB Full-Featured Type-C Receptacle connector</t>
+  </si>
+  <si>
+    <t>Amphenol Commercial Products</t>
+  </si>
+  <si>
+    <t>12401610E4#2A</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>X608</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <t>https://www.buydisplay.com/download/manual/ER-TFT1.28-2_Datasheet.pdf</t>
+  </si>
+  <si>
+    <t>ER-CON0.4-24P</t>
+  </si>
+  <si>
+    <t>EastRising</t>
+  </si>
+  <si>
+    <t>OK-24F024-04</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>X701 X702</t>
+  </si>
+  <si>
+    <t>MB1</t>
+  </si>
+  <si>
+    <t>https://cdn.amphenol-cs.com/media/wysiwyg/files/drawing/101r014fb110.pdf</t>
+  </si>
+  <si>
+    <t>101R014FB110</t>
+  </si>
+  <si>
+    <t>Generic connector, double row, 02x07, top/bottom pin numbering scheme (row 1: 1...pins_per_row, row2: pins_per_row+1 ... num_pins), script generated (kicad-library-utils/schlib/autogen/connector/)</t>
+  </si>
+  <si>
+    <t>Amphenol Aorora</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>X509</t>
+  </si>
+  <si>
+    <t>Motor</t>
+  </si>
+  <si>
+    <t>https://www.molex.com/en-us/products/part-detail-pdf/781710002?display=pdf</t>
+  </si>
+  <si>
+    <t>78171-0002</t>
   </si>
   <si>
     <t>Generic connector, single row, 01x02, script generated (kicad-library-utils/schlib/autogen/connector/)</t>
   </si>
   <si>
-    <t>JST Commercial</t>
-  </si>
-  <si>
-    <t>SM02B-SRSS-TB</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>X603</t>
-  </si>
-  <si>
-    <t>Device</t>
-  </si>
-  <si>
-    <t>https://www.usb.org/sites/default/files/documents/usb_type-c.zip</t>
-  </si>
-  <si>
-    <t>USB_C_Receptacle_Amphenol_12401610E4-2A</t>
-  </si>
-  <si>
-    <t>USB Full-Featured Type-C Receptacle connector</t>
-  </si>
-  <si>
-    <t>Amphenol Commercial Products</t>
-  </si>
-  <si>
-    <t>12401610E4#2A</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>X608</t>
-  </si>
-  <si>
-    <t>Display</t>
-  </si>
-  <si>
-    <t>https://www.buydisplay.com/download/manual/ER-TFT1.28-2_Datasheet.pdf</t>
-  </si>
-  <si>
-    <t>ER-CON0.4-24P</t>
-  </si>
-  <si>
-    <t>EastRising</t>
-  </si>
-  <si>
-    <t>OK-24F024-04</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>X701 X702</t>
-  </si>
-  <si>
-    <t>MB1</t>
-  </si>
-  <si>
-    <t>https://cdn.amphenol-cs.com/media/wysiwyg/files/drawing/101r014fb110.pdf</t>
-  </si>
-  <si>
-    <t>101R014FB110</t>
-  </si>
-  <si>
-    <t>Generic connector, double row, 02x07, top/bottom pin numbering scheme (row 1: 1...pins_per_row, row2: pins_per_row+1 ... num_pins), script generated (kicad-library-utils/schlib/autogen/connector/)</t>
-  </si>
-  <si>
-    <t>Amphenol Aorora</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>X509</t>
-  </si>
-  <si>
-    <t>Motor</t>
-  </si>
-  <si>
-    <t>https://www.molex.com/en-us/products/part-detail-pdf/781710002?display=pdf</t>
-  </si>
-  <si>
-    <t>78171-0002</t>
-  </si>
-  <si>
     <t>Molex</t>
   </si>
   <si>
@@ -995,7 +992,7 @@
     <t>Component Count:</t>
   </si>
   <si>
-    <t>62 (58 SMD/ 4 THT)</t>
+    <t>62 (57 SMD/ 4 THT)</t>
   </si>
   <si>
     <t>Fitted Components:</t>
@@ -1061,10 +1058,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-02-20 15:50:37</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.5</t>
+    <t>2026-09-04 19:37:04</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.21 + KiBot v1.9.1</t>
   </si>
   <si>
     <t>Columns colors</t>
@@ -1812,7 +1809,7 @@
     <col min="3" max="3" width="60.7109375" customWidth="1"/>
     <col min="4" max="4" width="21.7109375" customWidth="1"/>
     <col min="5" max="5" width="60.7109375" customWidth="1"/>
-    <col min="6" max="6" width="53.7109375" customWidth="1"/>
+    <col min="6" max="6" width="52.7109375" customWidth="1"/>
     <col min="7" max="7" width="60.7109375" customWidth="1"/>
     <col min="8" max="8" width="33.7109375" customWidth="1"/>
     <col min="9" max="9" width="37.7109375" customWidth="1"/>
@@ -1820,7 +1817,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="32" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1833,13 +1830,13 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="C2" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D2" s="3">
         <v>37</v>
@@ -1847,41 +1844,41 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>226</v>
-      </c>
       <c r="C3" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>233</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>229</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
@@ -1889,13 +1886,13 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>231</v>
-      </c>
       <c r="C6" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D6" s="3">
         <v>62</v>
@@ -2452,33 +2449,33 @@
         <v>116</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" ht="45" customHeight="1">
       <c r="A27" s="5" t="s">
         <v>117</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>118</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>28</v>
+        <v>119</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I27" s="7" t="s">
         <v>122</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -2486,28 +2483,28 @@
         <v>123</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>124</v>
       </c>
       <c r="D28" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="F28" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="G28" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="G28" s="10" t="s">
-        <v>125</v>
-      </c>
       <c r="H28" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -2527,19 +2524,19 @@
         <v>132</v>
       </c>
       <c r="F29" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="G29" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="G29" s="12" t="s">
-        <v>54</v>
-      </c>
       <c r="H29" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="I29" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="30" customHeight="1">
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" s="8" t="s">
         <v>135</v>
       </c>
@@ -2558,14 +2555,14 @@
       <c r="F30" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="G30" s="10" t="s">
+      <c r="G30" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H30" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="I30" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="30" customHeight="1">
@@ -2573,7 +2570,7 @@
         <v>141</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>142</v>
@@ -2585,422 +2582,422 @@
         <v>144</v>
       </c>
       <c r="F31" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G31" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="G31" s="7" t="s">
+      <c r="H31" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="H31" s="7" t="s">
-        <v>147</v>
-      </c>
       <c r="I31" s="7" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="30" customHeight="1">
       <c r="A32" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B32" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="E32" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="F32" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="E32" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>145</v>
-      </c>
       <c r="G32" s="10" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="30" customHeight="1">
       <c r="A33" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H33" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="H33" s="7" t="s">
-        <v>147</v>
-      </c>
       <c r="I33" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="30" customHeight="1">
       <c r="A34" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="30" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="30" customHeight="1">
       <c r="A36" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="30" customHeight="1">
       <c r="A37" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="G37" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I37" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="I37" s="7" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="30" customHeight="1">
       <c r="A38" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B38" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C38" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="E38" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="F38" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="E38" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>173</v>
-      </c>
       <c r="G38" s="10" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="30" customHeight="1">
       <c r="A39" s="5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C39" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H39" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="I39" s="7" t="s">
         <v>182</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="30" customHeight="1">
       <c r="A40" s="8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B40" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="30" customHeight="1">
       <c r="A41" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="I41" s="7" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="30" customHeight="1">
       <c r="A42" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B42" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C42" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E42" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="F42" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="G42" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="H42" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="G42" s="10" t="s">
+      <c r="I42" s="10" t="s">
         <v>199</v>
-      </c>
-      <c r="H42" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="I42" s="10" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="30" customHeight="1">
       <c r="A43" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C43" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="F43" s="6" t="s">
         <v>204</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>206</v>
       </c>
       <c r="G43" s="12" t="s">
         <v>54</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="I43" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="60" customHeight="1">
       <c r="A44" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B44" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C44" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="E44" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="D44" s="9" t="s">
+      <c r="F44" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="G44" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="F44" s="9" t="s">
+      <c r="H44" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="G44" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="H44" s="10" t="s">
-        <v>215</v>
-      </c>
       <c r="I44" s="10" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="30" customHeight="1">
       <c r="A45" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C45" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="F45" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="E45" s="6" t="s">
+      <c r="G45" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="F45" s="6" t="s">
+      <c r="H45" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G45" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>221</v>
-      </c>
       <c r="I45" s="7" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -3058,9 +3055,9 @@
   <cols>
     <col min="1" max="1" width="60.7109375" customWidth="1"/>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.7109375" customWidth="1" outlineLevel="2"/>
+    <col min="3" max="3" width="48.7109375" customWidth="1" outlineLevel="2"/>
     <col min="4" max="4" width="29.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="33.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="51.7109375" customWidth="1" outlineLevel="1"/>
     <col min="6" max="6" width="17.7109375" customWidth="1" outlineLevel="1"/>
     <col min="7" max="7" width="22.7109375" customWidth="1"/>
     <col min="8" max="8" width="16.7109375" customWidth="1"/>
@@ -3074,7 +3071,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="32" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3086,13 +3083,13 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="G2" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H2" s="13">
         <v>1</v>
@@ -3100,13 +3097,13 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>226</v>
-      </c>
       <c r="G3" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H3" s="15">
         <f>TotalCost/BoardQty</f>
@@ -3115,13 +3112,13 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H4" s="16">
         <f>SUM(H10:H46)</f>
@@ -3138,23 +3135,23 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>230</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="18" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B8" s="18"/>
       <c r="C8" s="18"/>
@@ -3164,7 +3161,7 @@
       <c r="G8" s="18"/>
       <c r="H8" s="18"/>
       <c r="I8" s="19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J8" s="19"/>
       <c r="K8" s="19"/>
@@ -3183,37 +3180,37 @@
         <v>5</v>
       </c>
       <c r="D9" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="E9" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="F9" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="G9" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="H9" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="H9" s="20" t="s">
-        <v>243</v>
-      </c>
       <c r="I9" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="J9" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="J9" s="20" t="s">
+      <c r="K9" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="L9" s="20" t="s">
         <v>246</v>
       </c>
-      <c r="K9" s="20" t="s">
+      <c r="M9" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="L9" s="20" t="s">
+      <c r="N9" s="20" t="s">
         <v>247</v>
-      </c>
-      <c r="M9" s="20" t="s">
-        <v>243</v>
-      </c>
-      <c r="N9" s="20" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="30" customHeight="1">
@@ -3743,20 +3740,17 @@
         <v>118</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>28</v>
+        <v>119</v>
       </c>
       <c r="C28" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="D28" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>122</v>
-      </c>
       <c r="F28" s="21">
-        <f>CEILING(BoardQty*2,1)</f>
-        <v>2</v>
+        <f>BoardQty*1</f>
+        <v>1</v>
       </c>
       <c r="G28" s="22">
         <f>IF(MIN(K28)&lt;&gt;0,MIN(K28),"")</f>
@@ -3772,20 +3766,20 @@
         <v>124</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>125</v>
+        <v>28</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D29" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="E29" s="21" t="s">
-        <v>127</v>
-      </c>
       <c r="F29" s="21">
-        <f>BoardQty*1</f>
-        <v>1</v>
+        <f>CEILING(BoardQty*2,1)</f>
+        <v>2</v>
       </c>
       <c r="G29" s="22">
         <f>IF(MIN(K29)&lt;&gt;0,MIN(K29),"")</f>
@@ -3804,13 +3798,13 @@
         <v>131</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D30" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="E30" s="21" t="s">
         <v>133</v>
-      </c>
-      <c r="E30" s="21" t="s">
-        <v>134</v>
       </c>
       <c r="F30" s="21">
         <f>BoardQty*1</f>
@@ -3836,10 +3830,10 @@
         <v>137</v>
       </c>
       <c r="D31" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="E31" s="21" t="s">
         <v>140</v>
-      </c>
-      <c r="E31" s="21" t="s">
-        <v>137</v>
       </c>
       <c r="F31" s="21">
         <f>BoardQty*1</f>
@@ -3862,17 +3856,17 @@
         <v>143</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F32" s="21">
-        <f>CEILING(BoardQty*2,1)</f>
-        <v>2</v>
+        <f>BoardQty*1</f>
+        <v>1</v>
       </c>
       <c r="G32" s="22">
         <f>IF(MIN(K32)&lt;&gt;0,MIN(K32),"")</f>
@@ -3885,19 +3879,19 @@
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="21" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B33" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="C33" s="21" t="s">
-        <v>145</v>
-      </c>
       <c r="D33" s="21" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E33" s="21" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F33" s="21">
         <f>CEILING(BoardQty*2,1)</f>
@@ -3914,23 +3908,23 @@
     </row>
     <row r="34" spans="1:13">
       <c r="A34" s="21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D34" s="21" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F34" s="21">
-        <f>BoardQty*1</f>
-        <v>1</v>
+        <f>CEILING(BoardQty*2,1)</f>
+        <v>2</v>
       </c>
       <c r="G34" s="22">
         <f>IF(MIN(K34)&lt;&gt;0,MIN(K34),"")</f>
@@ -3943,19 +3937,19 @@
     </row>
     <row r="35" spans="1:13">
       <c r="A35" s="21" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C35" s="21" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D35" s="21" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E35" s="21" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F35" s="21">
         <f>BoardQty*1</f>
@@ -3972,53 +3966,53 @@
     </row>
     <row r="36" spans="1:13">
       <c r="A36" s="21" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F36" s="21">
+        <f>BoardQty*1</f>
+        <v>1</v>
+      </c>
+      <c r="G36" s="22">
+        <f>IF(MIN(K36)&lt;&gt;0,MIN(K36),"")</f>
+        <v/>
+      </c>
+      <c r="H36" s="23">
+        <f>IF(AND(ISNUMBER(F36),ISNUMBER(G36)),F36*G36,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="D37" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="E37" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="F37" s="21">
         <f>CEILING(BoardQty*2,1)</f>
         <v>2</v>
       </c>
-      <c r="G36" s="22">
-        <f>IF(MIN(K36)&lt;&gt;0,MIN(K36),"")</f>
-        <v/>
-      </c>
-      <c r="H36" s="23">
-        <f>IF(AND(ISNUMBER(F36),ISNUMBER(G36)),F36*G36,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="1:13">
-      <c r="A37" s="21" t="s">
-        <v>166</v>
-      </c>
-      <c r="B37" s="21" t="s">
-        <v>167</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>145</v>
-      </c>
-      <c r="D37" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="E37" s="21" t="s">
-        <v>168</v>
-      </c>
-      <c r="F37" s="21">
-        <f>BoardQty*1</f>
-        <v>1</v>
-      </c>
       <c r="G37" s="22">
         <f>IF(MIN(K37)&lt;&gt;0,MIN(K37),"")</f>
         <v/>
@@ -4030,19 +4024,19 @@
     </row>
     <row r="38" spans="1:13">
       <c r="A38" s="21" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>175</v>
+        <v>153</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F38" s="21">
         <f>BoardQty*1</f>
@@ -4059,19 +4053,19 @@
     </row>
     <row r="39" spans="1:13">
       <c r="A39" s="21" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B39" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="C39" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="C39" s="21" t="s">
-        <v>173</v>
-      </c>
       <c r="D39" s="21" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="F39" s="21">
         <f>BoardQty*1</f>
@@ -4088,19 +4082,19 @@
     </row>
     <row r="40" spans="1:13">
       <c r="A40" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="D40" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="E40" s="21" t="s">
         <v>182</v>
-      </c>
-      <c r="C40" s="21" t="s">
-        <v>173</v>
-      </c>
-      <c r="D40" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="E40" s="21" t="s">
-        <v>176</v>
       </c>
       <c r="F40" s="21">
         <f>BoardQty*1</f>
@@ -4117,19 +4111,19 @@
     </row>
     <row r="41" spans="1:13">
       <c r="A41" s="21" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D41" s="21" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="F41" s="21">
         <f>BoardQty*1</f>
@@ -4146,19 +4140,19 @@
     </row>
     <row r="42" spans="1:13">
       <c r="A42" s="21" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D42" s="21" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="F42" s="21">
         <f>BoardQty*1</f>
@@ -4175,19 +4169,19 @@
     </row>
     <row r="43" spans="1:13">
       <c r="A43" s="21" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B43" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="C43" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="C43" s="21" t="s">
+      <c r="D43" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="D43" s="21" t="s">
-        <v>200</v>
-      </c>
       <c r="E43" s="21" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F43" s="21">
         <f>BoardQty*1</f>
@@ -4204,19 +4198,19 @@
     </row>
     <row r="44" spans="1:13">
       <c r="A44" s="21" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B44" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="C44" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="C44" s="21" t="s">
+      <c r="D44" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="E44" s="21" t="s">
         <v>206</v>
-      </c>
-      <c r="D44" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="E44" s="21" t="s">
-        <v>208</v>
       </c>
       <c r="F44" s="21">
         <f>BoardQty*1</f>
@@ -4233,19 +4227,19 @@
     </row>
     <row r="45" spans="1:13">
       <c r="A45" s="21" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B45" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="C45" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="C45" s="21" t="s">
+      <c r="D45" s="21" t="s">
         <v>213</v>
       </c>
-      <c r="D45" s="21" t="s">
-        <v>215</v>
-      </c>
       <c r="E45" s="21" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F45" s="21">
         <f>CEILING(BoardQty*2,1)</f>
@@ -4262,19 +4256,19 @@
     </row>
     <row r="46" spans="1:13">
       <c r="A46" s="21" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B46" s="21" t="s">
+        <v>216</v>
+      </c>
+      <c r="C46" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="C46" s="21" t="s">
+      <c r="D46" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="D46" s="21" t="s">
-        <v>221</v>
-      </c>
       <c r="E46" s="21" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F46" s="21">
         <f>BoardQty*1</f>
@@ -4291,14 +4285,14 @@
     </row>
     <row r="48" spans="1:13">
       <c r="G48" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H48" s="16">
         <f>SUM(M48)</f>
         <v>0</v>
       </c>
       <c r="I48" s="24" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J48" s="17">
         <f>IFERROR(IF(COUNTIF(J10:J46,"&gt;0")&gt;0,COUNTIF(J10:J46,"&gt;0")&amp;" of "&amp;(ROWS(L10:L46)-COUNTBLANK(L10:L46))&amp;" parts purchased",""),"")</f>
@@ -4311,13 +4305,13 @@
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="B49" s="26" t="s">
         <v>255</v>
       </c>
-      <c r="B49" s="26" t="s">
-        <v>256</v>
-      </c>
       <c r="G49" s="27" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J49" s="28">
         <f>CONCATENATE(J87,J88,J89,J90,J91,J92,J93,J94,J95,J96,J97,J98,J99,J100,J101,J102,J103,J104,J105,J106,J107,J108,J109,J110,J111,J112,J113,J114,J115,J116,J117,J118,J119,J120,J121,J122,J123)</f>
@@ -4326,13 +4320,13 @@
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="29" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="87" spans="10:10" ht="30" hidden="1" customHeight="1">
       <c r="J87" t="str">
         <f t="array" ref="J87:J123">IF(ISNUMBER(J10:J46)*(J10:J46&gt;=L10:L46)*(N10:N46&lt;&gt;""),N10:N46&amp;"|"&amp;TEXT(ROUNDUP(J10:J46/IF(ISNUMBER(L10:L46),L10:L46,1),0)*L10:L46,"##0")&amp;"|"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(PURCHASE_DESCRIPTION&lt;&gt;"",PURCHASE_DESCRIPTION&amp;":","")&amp;A10:A46,"|",";")," ","_"),"
-","_")&amp;CHAR(10),"")</f>
+","_")&amp;CHAR(13),"")</f>
         <v/>
       </c>
     </row>
@@ -5096,77 +5090,77 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="30" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="31" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="32" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="33" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="34" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="35" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="37" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="38" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>